<commit_message>
update multiple files in revision
</commit_message>
<xml_diff>
--- a/01_Introduction_to_Data_Analytics/Mini_Project_The_Profitable_Car_Showroom.xlsx
+++ b/01_Introduction_to_Data_Analytics/Mini_Project_The_Profitable_Car_Showroom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 COURSES\Learn_Data_Analytics_by_CWH\01_Introduction_to_Data_Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB7BEB2-E580-4CCF-B522-95431EFD00F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D915C99-5D3D-452A-ABC2-865D0AF1C578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0EE9ECE5-E58C-432A-BD20-A3230641CDEF}"/>
   </bookViews>
@@ -452,16 +452,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D069564-1BC3-42E6-82D9-32C4FFDF040D}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="19" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1796875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -474,8 +475,9 @@
       <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -488,8 +490,9 @@
       <c r="D2" s="5">
         <v>3750000</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -502,8 +505,9 @@
       <c r="D3" s="5">
         <v>7600000</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -516,8 +520,9 @@
       <c r="D4" s="5">
         <v>6600000</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -530,8 +535,9 @@
       <c r="D5" s="6">
         <v>11250000</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -544,8 +550,9 @@
       <c r="D6" s="5">
         <v>6500000</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E6" s="1"/>
+    </row>
+    <row r="8" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="1">
         <f xml:space="preserve"> MAX(D2:D6)</f>
         <v>11250000</v>

</xml_diff>